<commit_message>
hardware: update DBA/DBB/FCU STR fab files to V1.0 (2026-06-13)
Refresh BOM, CPL, Gerber, schematic PDF and STEP for all three
boards from the 2026-06-13 fab package. Add Assembly_STEP/ with
full-assembly STEP models (DBA, DBB, FCU PRO, FCU STR).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DaugtherBoard_BCGA/BOM DBA.xlsx
+++ b/DaugtherBoard_BCGA/BOM DBA.xlsx
@@ -91,19 +91,19 @@
     <t>3</t>
   </si>
   <si>
-    <t>SH1.0mm-2P-LT</t>
-  </si>
-  <si>
-    <t>CN6,CN9,CN10,CN11</t>
-  </si>
-  <si>
-    <t>CONN-SMD_SH1.0MM-2P-LT</t>
-  </si>
-  <si>
-    <t>LXWCONN(连兴旺电子)</t>
-  </si>
-  <si>
-    <t>C53055327</t>
+    <t>S2B-ZR-SM2-TF(LF)(SN)</t>
+  </si>
+  <si>
+    <t>CN6,CN10,CN11</t>
+  </si>
+  <si>
+    <t>CONN-SMD_2P-P1.50_S2B-ZR-SM2-TF-LF-SN</t>
+  </si>
+  <si>
+    <t>JST</t>
+  </si>
+  <si>
+    <t>C5306678</t>
   </si>
   <si>
     <t>4</t>
@@ -115,16 +115,16 @@
     <t>R1,R2</t>
   </si>
   <si>
-    <t>R0603</t>
-  </si>
-  <si>
-    <t>FRC0603J102 TS</t>
-  </si>
-  <si>
-    <t>FOJAN(富捷)</t>
-  </si>
-  <si>
-    <t>C2907113</t>
+    <t>R1206</t>
+  </si>
+  <si>
+    <t>1206W4F1001T5E</t>
+  </si>
+  <si>
+    <t>UNI-ROYAL(厚声)</t>
+  </si>
+  <si>
+    <t>C4410</t>
   </si>
   <si>
     <t>5</t>
@@ -626,7 +626,7 @@
         <v>25</v>
       </c>
       <c r="B4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C4" t="s">
         <v>26</v>

</xml_diff>